<commit_message>
Updated AP3 Informationsmodell changes
</commit_message>
<xml_diff>
--- a/site/StructureDefinition-KBV-EX-WEST-Begegnung-Spezielle-Begegnungsinformationen.xlsx
+++ b/site/StructureDefinition-KBV-EX-WEST-Begegnung-Spezielle-Begegnungsinformationen.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="168">
   <si>
     <t>Property</t>
   </si>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-29T11:10:04+02:00</t>
+    <t>2026-06-24T16:51:19+02:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -78,7 +78,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Zusatzinformationen zur Begegnung, die nicht durch die regulären Encounter-Elemente oder durch andere fachliche Profile abgebildet werden. Sie dient der Erhaltung encounter-bezogener Kontextinformationen, insbesondere, wenn ein Inhalt eine Begegnung referenziert werden muss, um technisch valide zu sein, aber fachlich keine Begegnung zugeordnet werden kann. In diesem Fall ist die Instanz der Begegnung eine Dummy-Begegnung sein, mit der Extension „spezielle Begegnungsinformationen“ und folgenden Inhalt: Typ = Dummy Inhalt = Dummy</t>
+    <t>Spezielle Begegnungsinformationen</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -256,9 +256,6 @@
 </t>
   </si>
   <si>
-    <t>Spezielle Begegnungsinformationen</t>
-  </si>
-  <si>
     <t xml:space="preserve">ele-1
 </t>
   </si>
@@ -315,31 +312,25 @@
     <t>Element.extension</t>
   </si>
   <si>
-    <t>Extension.extension:typ</t>
-  </si>
-  <si>
-    <t>typ</t>
-  </si>
-  <si>
-    <t>Typ</t>
-  </si>
-  <si>
-    <t>Bezeichnung des Typs des Eintrags in der Begegnungsdokumentation. Teilweise auch bekannt als freie Kategorie</t>
-  </si>
-  <si>
-    <t>Extension.extension:typ.id</t>
+    <t>Extension.extension:schein-ID</t>
+  </si>
+  <si>
+    <t>schein-ID</t>
+  </si>
+  <si>
+    <t>Extension.extension:schein-ID.id</t>
   </si>
   <si>
     <t>Extension.extension.id</t>
   </si>
   <si>
-    <t>Extension.extension:typ.extension</t>
+    <t>Extension.extension:schein-ID.extension</t>
   </si>
   <si>
     <t>Extension.extension.extension</t>
   </si>
   <si>
-    <t>Extension.extension:typ.url</t>
+    <t>Extension.extension:schein-ID.url</t>
   </si>
   <si>
     <t>Extension.extension.url</t>
@@ -364,36 +355,66 @@
     <t>N/A</t>
   </si>
   <si>
+    <t>Extension.extension:schein-ID.value[x]</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x]</t>
+  </si>
+  <si>
+    <t>Value of extension</t>
+  </si>
+  <si>
+    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">type:$this}
+</t>
+  </si>
+  <si>
+    <t>closed</t>
+  </si>
+  <si>
+    <t>Extension.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+</t>
+  </si>
+  <si>
+    <t>Extension.extension:schein-ID.value[x]:valueString</t>
+  </si>
+  <si>
+    <t>valueString</t>
+  </si>
+  <si>
+    <t>Extension.extension:typ</t>
+  </si>
+  <si>
+    <t>typ</t>
+  </si>
+  <si>
+    <t>Typ</t>
+  </si>
+  <si>
+    <t>Bezeichnung des Typs des Eintrags in der Begegnungsdokumentation. Teilweise auch bekannt als freie Kategorie</t>
+  </si>
+  <si>
+    <t>Extension.extension:typ.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:typ.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:typ.url</t>
+  </si>
+  <si>
     <t>Extension.extension:typ.value[x]</t>
-  </si>
-  <si>
-    <t>Extension.extension.value[x]</t>
   </si>
   <si>
     <t xml:space="preserve">CodeableConcept
 </t>
   </si>
   <si>
-    <t>Value of extension</t>
-  </si>
-  <si>
-    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type:$this}
-</t>
-  </si>
-  <si>
-    <t>closed</t>
-  </si>
-  <si>
-    <t>Extension.value[x]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-</t>
-  </si>
-  <si>
     <t>Extension.extension:typ.value[x]:valueCodeableConcept</t>
   </si>
   <si>
@@ -505,9 +526,6 @@
   </si>
   <si>
     <t>Extension.extension:inhalt.value[x]:valueString</t>
-  </si>
-  <si>
-    <t>valueString</t>
   </si>
   <si>
     <t>base64Binary
@@ -823,7 +841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK22"/>
+  <dimension ref="A1:AK28"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="54.3515625" customWidth="true" bestFit="true"/>
@@ -1008,7 +1026,7 @@
         <v>79</v>
       </c>
       <c r="L2" t="s" s="2">
-        <v>80</v>
+        <v>21</v>
       </c>
       <c r="M2" t="s" s="2">
         <v>21</v>
@@ -1071,10 +1089,10 @@
         <v>78</v>
       </c>
       <c r="AI2" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ2" t="s" s="2">
         <v>81</v>
-      </c>
-      <c r="AJ2" t="s" s="2">
-        <v>82</v>
       </c>
       <c r="AK2" t="s" s="2">
         <v>76</v>
@@ -1082,10 +1100,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" t="s" s="2">
@@ -1096,25 +1114,25 @@
         <v>77</v>
       </c>
       <c r="G3" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H3" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I3" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J3" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K3" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="H3" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I3" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J3" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K3" t="s" s="2">
+      <c r="L3" t="s" s="2">
         <v>85</v>
       </c>
-      <c r="L3" t="s" s="2">
+      <c r="M3" t="s" s="2">
         <v>86</v>
-      </c>
-      <c r="M3" t="s" s="2">
-        <v>87</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -1165,30 +1183,30 @@
         <v>76</v>
       </c>
       <c r="AF3" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AG3" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH3" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI3" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ3" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK3" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="AG3" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH3" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI3" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ3" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK3" t="s" s="2">
-        <v>89</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" t="s" s="2">
@@ -1196,7 +1214,7 @@
       </c>
       <c r="E4" s="2"/>
       <c r="F4" t="s" s="2">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G4" t="s" s="2">
         <v>78</v>
@@ -1211,13 +1229,13 @@
         <v>76</v>
       </c>
       <c r="K4" t="s" s="2">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L4" t="s" s="2">
         <v>30</v>
       </c>
       <c r="M4" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -1256,19 +1274,19 @@
         <v>76</v>
       </c>
       <c r="AB4" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AC4" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="AC4" t="s" s="2">
+      <c r="AD4" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE4" t="s" s="2">
         <v>95</v>
       </c>
-      <c r="AD4" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE4" t="s" s="2">
+      <c r="AF4" t="s" s="2">
         <v>96</v>
-      </c>
-      <c r="AF4" t="s" s="2">
-        <v>97</v>
       </c>
       <c r="AG4" t="s" s="2">
         <v>77</v>
@@ -1277,10 +1295,10 @@
         <v>78</v>
       </c>
       <c r="AI4" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ4" t="s" s="2">
         <v>81</v>
-      </c>
-      <c r="AJ4" t="s" s="2">
-        <v>82</v>
       </c>
       <c r="AK4" t="s" s="2">
         <v>76</v>
@@ -1288,23 +1306,23 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="C5" t="s" s="2">
         <v>98</v>
-      </c>
-      <c r="B5" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>99</v>
       </c>
       <c r="D5" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G5" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H5" t="s" s="2">
         <v>76</v>
@@ -1316,13 +1334,13 @@
         <v>76</v>
       </c>
       <c r="K5" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="L5" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="M5" t="s" s="2">
         <v>92</v>
-      </c>
-      <c r="L5" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="M5" t="s" s="2">
-        <v>101</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1373,7 +1391,7 @@
         <v>76</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>77</v>
@@ -1382,10 +1400,10 @@
         <v>78</v>
       </c>
       <c r="AI5" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ5" t="s" s="2">
         <v>81</v>
-      </c>
-      <c r="AJ5" t="s" s="2">
-        <v>82</v>
       </c>
       <c r="AK5" t="s" s="2">
         <v>76</v>
@@ -1393,10 +1411,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1407,25 +1425,25 @@
         <v>77</v>
       </c>
       <c r="G6" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K6" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="H6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K6" t="s" s="2">
+      <c r="L6" t="s" s="2">
         <v>85</v>
       </c>
-      <c r="L6" t="s" s="2">
+      <c r="M6" t="s" s="2">
         <v>86</v>
-      </c>
-      <c r="M6" t="s" s="2">
-        <v>87</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -1476,30 +1494,30 @@
         <v>76</v>
       </c>
       <c r="AF6" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AG6" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH6" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK6" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="AG6" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH6" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK6" t="s" s="2">
-        <v>89</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1522,13 +1540,13 @@
         <v>76</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L7" t="s" s="2">
         <v>30</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1567,19 +1585,19 @@
         <v>76</v>
       </c>
       <c r="AB7" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AC7" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="AC7" t="s" s="2">
+      <c r="AD7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE7" t="s" s="2">
         <v>95</v>
       </c>
-      <c r="AD7" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE7" t="s" s="2">
+      <c r="AF7" t="s" s="2">
         <v>96</v>
-      </c>
-      <c r="AF7" t="s" s="2">
-        <v>97</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>77</v>
@@ -1588,10 +1606,10 @@
         <v>78</v>
       </c>
       <c r="AI7" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ7" t="s" s="2">
         <v>81</v>
-      </c>
-      <c r="AJ7" t="s" s="2">
-        <v>82</v>
       </c>
       <c r="AK7" t="s" s="2">
         <v>76</v>
@@ -1599,10 +1617,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1610,10 +1628,10 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H8" t="s" s="2">
         <v>76</v>
@@ -1625,16 +1643,16 @@
         <v>76</v>
       </c>
       <c r="K8" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="L8" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="M8" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="N8" t="s" s="2">
         <v>108</v>
-      </c>
-      <c r="L8" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="M8" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="N8" t="s" s="2">
-        <v>111</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1642,7 +1660,7 @@
       </c>
       <c r="Q8" s="2"/>
       <c r="R8" t="s" s="2">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="S8" t="s" s="2">
         <v>76</v>
@@ -1684,13 +1702,13 @@
         <v>76</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="AG8" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AH8" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AI8" t="s" s="2">
         <v>76</v>
@@ -1699,15 +1717,15 @@
         <v>76</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1715,28 +1733,28 @@
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G9" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H9" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I9" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J9" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K9" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="G9" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H9" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I9" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J9" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K9" t="s" s="2">
-        <v>116</v>
-      </c>
       <c r="L9" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1775,71 +1793,71 @@
         <v>76</v>
       </c>
       <c r="AB9" t="s" s="2">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="AC9" s="2"/>
       <c r="AD9" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE9" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH9" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AI9" t="s" s="2">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G10" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H10" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I10" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J10" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K10" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="G10" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H10" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I10" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J10" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K10" t="s" s="2">
-        <v>116</v>
-      </c>
       <c r="L10" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1890,41 +1908,43 @@
         <v>76</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH10" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="AK10" t="s" s="2">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>126</v>
-      </c>
-      <c r="C11" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="C11" t="s" s="2">
+        <v>122</v>
+      </c>
       <c r="D11" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G11" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H11" t="s" s="2">
         <v>76</v>
@@ -1936,13 +1956,13 @@
         <v>76</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>86</v>
+        <v>123</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -1993,41 +2013,41 @@
         <v>76</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH11" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AI11" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AK11" t="s" s="2">
-        <v>89</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
-        <v>129</v>
+        <v>76</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>76</v>
@@ -2039,17 +2059,15 @@
         <v>76</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>130</v>
+        <v>85</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="N12" t="s" s="2">
-        <v>132</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
         <v>76</v>
@@ -2086,42 +2104,42 @@
         <v>76</v>
       </c>
       <c r="AB12" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC12" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD12" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE12" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH12" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI12" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AK12" t="s" s="2">
-        <v>113</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>134</v>
+        <v>102</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2132,7 +2150,7 @@
         <v>77</v>
       </c>
       <c r="G13" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H13" t="s" s="2">
         <v>76</v>
@@ -2141,23 +2159,19 @@
         <v>76</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>135</v>
+        <v>76</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>136</v>
+        <v>91</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>137</v>
+        <v>30</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="N13" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="O13" t="s" s="2">
-        <v>140</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
         <v>76</v>
       </c>
@@ -2193,19 +2207,19 @@
         <v>76</v>
       </c>
       <c r="AB13" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AC13" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AD13" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE13" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>141</v>
+        <v>96</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>77</v>
@@ -2214,21 +2228,21 @@
         <v>78</v>
       </c>
       <c r="AI13" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ13" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="AJ13" t="s" s="2">
-        <v>122</v>
-      </c>
       <c r="AK13" t="s" s="2">
-        <v>142</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>144</v>
+        <v>104</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2236,10 +2250,10 @@
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G14" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H14" t="s" s="2">
         <v>76</v>
@@ -2248,29 +2262,27 @@
         <v>76</v>
       </c>
       <c r="J14" t="s" s="2">
-        <v>135</v>
+        <v>76</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>146</v>
+        <v>107</v>
       </c>
       <c r="N14" t="s" s="2">
-        <v>147</v>
-      </c>
-      <c r="O14" t="s" s="2">
-        <v>148</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q14" s="2"/>
       <c r="R14" t="s" s="2">
-        <v>76</v>
+        <v>122</v>
       </c>
       <c r="S14" t="s" s="2">
         <v>76</v>
@@ -2312,43 +2324,41 @@
         <v>76</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>149</v>
+        <v>109</v>
       </c>
       <c r="AG14" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="AH14" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AI14" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>150</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="C15" t="s" s="2">
-        <v>152</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>76</v>
@@ -2360,13 +2370,13 @@
         <v>76</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>153</v>
+        <v>113</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2405,53 +2415,53 @@
         <v>76</v>
       </c>
       <c r="AB15" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC15" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="AC15" s="2"/>
       <c r="AD15" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE15" t="s" s="2">
-        <v>76</v>
+        <v>116</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH15" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI15" t="s" s="2">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>82</v>
+        <v>118</v>
       </c>
       <c r="AK15" t="s" s="2">
-        <v>76</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="C16" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="C16" t="s" s="2">
+        <v>131</v>
+      </c>
       <c r="D16" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H16" t="s" s="2">
         <v>76</v>
@@ -2463,13 +2473,13 @@
         <v>76</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>85</v>
+        <v>129</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>87</v>
+        <v>114</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2520,30 +2530,30 @@
         <v>76</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>88</v>
+        <v>117</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AI16" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ16" t="s" s="2">
-        <v>76</v>
+        <v>118</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>89</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>156</v>
+        <v>132</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>105</v>
+        <v>133</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2554,7 +2564,7 @@
         <v>77</v>
       </c>
       <c r="G17" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H17" t="s" s="2">
         <v>76</v>
@@ -2566,13 +2576,13 @@
         <v>76</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2611,53 +2621,53 @@
         <v>76</v>
       </c>
       <c r="AB17" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AC17" t="s" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="AD17" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE17" t="s" s="2">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH17" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI17" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AK17" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>107</v>
+        <v>135</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>76</v>
+        <v>136</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H18" t="s" s="2">
         <v>76</v>
@@ -2669,16 +2679,16 @@
         <v>76</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>109</v>
+        <v>137</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>110</v>
+        <v>138</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>111</v>
+        <v>139</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -2686,7 +2696,7 @@
       </c>
       <c r="Q18" s="2"/>
       <c r="R18" t="s" s="2">
-        <v>152</v>
+        <v>76</v>
       </c>
       <c r="S18" t="s" s="2">
         <v>76</v>
@@ -2716,42 +2726,42 @@
         <v>76</v>
       </c>
       <c r="AB18" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AC18" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AD18" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE18" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="AG18" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AH18" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AI18" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ18" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>115</v>
+        <v>141</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2759,10 +2769,10 @@
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G19" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H19" t="s" s="2">
         <v>76</v>
@@ -2771,19 +2781,23 @@
         <v>76</v>
       </c>
       <c r="J19" t="s" s="2">
-        <v>76</v>
+        <v>142</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>85</v>
+        <v>143</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>117</v>
+        <v>144</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
+        <v>145</v>
+      </c>
+      <c r="N19" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="O19" t="s" s="2">
+        <v>147</v>
+      </c>
       <c r="P19" t="s" s="2">
         <v>76</v>
       </c>
@@ -2819,74 +2833,78 @@
         <v>76</v>
       </c>
       <c r="AB19" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="AC19" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="AC19" t="s" s="2">
+        <v>76</v>
+      </c>
       <c r="AD19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE19" t="s" s="2">
-        <v>120</v>
+        <v>76</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>121</v>
+        <v>148</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH19" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AI19" t="s" s="2">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>113</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="C20" t="s" s="2">
-        <v>160</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G20" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J20" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="K20" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="G20" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H20" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I20" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J20" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K20" t="s" s="2">
-        <v>85</v>
-      </c>
       <c r="L20" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="M20" t="s" s="2">
         <v>153</v>
       </c>
-      <c r="M20" t="s" s="2">
+      <c r="N20" t="s" s="2">
         <v>154</v>
       </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
+      <c r="O20" t="s" s="2">
+        <v>155</v>
+      </c>
       <c r="P20" t="s" s="2">
         <v>76</v>
       </c>
@@ -2934,41 +2952,43 @@
         <v>76</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>121</v>
+        <v>156</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AI20" t="s" s="2">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>113</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>112</v>
+        <v>158</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="C21" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="C21" t="s" s="2">
+        <v>159</v>
+      </c>
       <c r="D21" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H21" t="s" s="2">
         <v>76</v>
@@ -2980,24 +3000,22 @@
         <v>76</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>109</v>
+        <v>160</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="N21" t="s" s="2">
-        <v>111</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q21" s="2"/>
       <c r="R21" t="s" s="2">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="S21" t="s" s="2">
         <v>76</v>
@@ -3039,30 +3057,30 @@
         <v>76</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="AG21" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AI21" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>113</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>121</v>
+        <v>162</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3073,7 +3091,7 @@
         <v>77</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>76</v>
@@ -3085,13 +3103,13 @@
         <v>76</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>161</v>
+        <v>84</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>117</v>
+        <v>85</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3142,22 +3160,644 @@
         <v>76</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>121</v>
+        <v>87</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH22" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK22" t="s" s="2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="B23" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G23" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K23" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="L23" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="M23" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="P23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q23" s="2"/>
+      <c r="R23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB23" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AC23" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AD23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE23" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AF23" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AG23" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH23" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI23" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ23" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK23" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="B24" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G24" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K24" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="L24" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="M24" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="N24" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="O24" s="2"/>
+      <c r="P24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q24" s="2"/>
+      <c r="R24" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="S24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF24" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AG24" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH24" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK24" t="s" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="B25" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G25" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K25" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="AI22" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ22" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="AK22" t="s" s="2">
+      <c r="L25" t="s" s="2">
         <v>113</v>
+      </c>
+      <c r="M25" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="N25" s="2"/>
+      <c r="O25" s="2"/>
+      <c r="P25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q25" s="2"/>
+      <c r="R25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB25" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AC25" s="2"/>
+      <c r="AD25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE25" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AF25" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="AG25" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH25" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ25" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="AK25" t="s" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="B26" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="C26" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="D26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G26" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K26" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="L26" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="M26" t="s" s="2">
+        <v>161</v>
+      </c>
+      <c r="N26" s="2"/>
+      <c r="O26" s="2"/>
+      <c r="P26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q26" s="2"/>
+      <c r="R26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF26" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="AG26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH26" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ26" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="AK26" t="s" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="B27" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G27" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K27" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="L27" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="M27" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="O27" s="2"/>
+      <c r="P27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q27" s="2"/>
+      <c r="R27" t="s" s="2">
+        <v>3</v>
+      </c>
+      <c r="S27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF27" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AG27" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH27" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK27" t="s" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="B28" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E28" s="2"/>
+      <c r="F28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K28" t="s" s="2">
+        <v>167</v>
+      </c>
+      <c r="L28" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="M28" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2"/>
+      <c r="P28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q28" s="2"/>
+      <c r="R28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF28" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="AG28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH28" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ28" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="AK28" t="s" s="2">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>